<commit_message>
Sync: Add/Update tbb-LPSCI folder - 2026-04-29 20:50
</commit_message>
<xml_diff>
--- a/tbb-LPSCI/all.xlsx
+++ b/tbb-LPSCI/all.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tbb-LPSCI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104961D5-B65B-46DF-8AFD-6D21F8BBEF6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB7AD4A-82A0-4FFB-94CE-DBF462A69FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lattice" sheetId="1" r:id="rId1"/>
+    <sheet name="formation" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="61">
   <si>
     <r>
       <t>Li</t>
@@ -298,6 +299,432 @@
   </si>
   <si>
     <t>supercell</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CldopingI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Iatom</t>
+  </si>
+  <si>
+    <t>I1</t>
+  </si>
+  <si>
+    <t>I-mp1525634</t>
+  </si>
+  <si>
+    <t>I8</t>
+  </si>
+  <si>
+    <t>I-mp23153</t>
+  </si>
+  <si>
+    <t>I-mp601148</t>
+  </si>
+  <si>
+    <t>I2</t>
+  </si>
+  <si>
+    <t>I-mp639715</t>
+  </si>
+  <si>
+    <t>I-mp684663</t>
+  </si>
+  <si>
+    <t>Cl2-mp1008394</t>
+  </si>
+  <si>
+    <t>Cl8</t>
+  </si>
+  <si>
+    <t>Cl2-mp22848</t>
+  </si>
+  <si>
+    <t>Cl2-mp570778</t>
+  </si>
+  <si>
+    <t>Cl16</t>
+  </si>
+  <si>
+    <t>Clatom</t>
+  </si>
+  <si>
+    <t>Cl1</t>
+  </si>
+  <si>
+    <t>Li2S-mp1125</t>
+  </si>
+  <si>
+    <t>Li8S4</t>
+  </si>
+  <si>
+    <t>Li2S-mp1153</t>
+  </si>
+  <si>
+    <t>Li2S-mp557142</t>
+  </si>
+  <si>
+    <t>Li4S2</t>
+  </si>
+  <si>
+    <t>Li2S-mp723352</t>
+  </si>
+  <si>
+    <t>Li22S11</t>
+  </si>
+  <si>
+    <t>LiCl-mp1185319</t>
+  </si>
+  <si>
+    <t>Li2Cl2</t>
+  </si>
+  <si>
+    <t>LiCl-mp22905</t>
+  </si>
+  <si>
+    <t>Li4Cl4</t>
+  </si>
+  <si>
+    <t>LiI-mp22899</t>
+  </si>
+  <si>
+    <t>Li4I4</t>
+  </si>
+  <si>
+    <t>LiI-mp568273</t>
+  </si>
+  <si>
+    <t>Li2I2</t>
+  </si>
+  <si>
+    <t>LiI-mp570935</t>
+  </si>
+  <si>
+    <t>P2S5-mp541788</t>
+  </si>
+  <si>
+    <t>P8S20</t>
+  </si>
+  <si>
+    <t>formation energy (eV/atom)</t>
+  </si>
+  <si>
+    <t>7 LiCl+ 4 P2S5 + 20 Li2S + LiI→Li48P8S40Cl7I1</t>
+  </si>
+  <si>
+    <t>文件夹</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>总能量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>计量比</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每化学式能量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Li</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>48</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cl</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Li</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>48</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cl</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>8</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CldopingI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Li48P8S40Cl8 - Cl + I → Li48P8S40Cl7I1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分子式</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分子式</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Li</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>24</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cl</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I0125-1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I0125-2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -361,11 +788,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,50 +1077,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:H9"/>
+  <dimension ref="A3:I10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.375" customWidth="1"/>
+    <col min="3" max="3" width="10.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>1</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>10.01233</v>
       </c>
-      <c r="D4">
-        <f>C4</f>
+      <c r="E4">
+        <f>D4</f>
         <v>10.01233</v>
       </c>
-      <c r="E4">
-        <f>C4</f>
+      <c r="F4">
+        <f>D4</f>
         <v>10.01233</v>
-      </c>
-      <c r="F4">
-        <v>90</v>
       </c>
       <c r="G4">
         <v>90</v>
@@ -698,24 +1129,27 @@
       <c r="H4">
         <v>90</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="I4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5">
         <v>9.8578150000000004</v>
       </c>
-      <c r="D5">
-        <f>C5</f>
+      <c r="E5">
+        <f>D5</f>
         <v>9.8578150000000004</v>
       </c>
-      <c r="E5">
-        <f>C5</f>
+      <c r="F5">
+        <f>D5</f>
         <v>9.8578150000000004</v>
-      </c>
-      <c r="F5">
-        <v>90</v>
       </c>
       <c r="G5">
         <v>90</v>
@@ -723,47 +1157,53 @@
       <c r="H5">
         <v>90</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B8" t="s">
         <v>0</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8">
         <v>10.01233</v>
       </c>
-      <c r="D8">
-        <f>C8</f>
+      <c r="E8">
+        <f>D8</f>
         <v>10.01233</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>20.024650000000001</v>
-      </c>
-      <c r="F8">
-        <v>90</v>
       </c>
       <c r="G8">
         <v>90</v>
@@ -771,29 +1211,64 @@
       <c r="H8">
         <v>90</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="I8">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9">
         <v>9.8186099999999996</v>
       </c>
-      <c r="D9">
-        <f>C9</f>
+      <c r="E9">
+        <f>D9</f>
         <v>9.8186099999999996</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>19.049389999999999</v>
-      </c>
-      <c r="F9">
-        <v>90</v>
       </c>
       <c r="G9">
         <v>90</v>
       </c>
       <c r="H9">
+        <v>90</v>
+      </c>
+      <c r="I9">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10">
+        <v>9.8100299999999994</v>
+      </c>
+      <c r="E10">
+        <v>9.8100299999999994</v>
+      </c>
+      <c r="F10">
+        <v>18.92792</v>
+      </c>
+      <c r="G10">
+        <v>90</v>
+      </c>
+      <c r="H10">
+        <v>90</v>
+      </c>
+      <c r="I10">
         <v>90</v>
       </c>
     </row>
@@ -805,4 +1280,533 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF08B60D-E41C-4BF4-A430-79D9B65D3070}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.875" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3">
+        <v>-0.20510769000000001</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3">
+        <v>-0.20510700000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3">
+        <v>-20.52960981</v>
+      </c>
+      <c r="D3" s="3">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3">
+        <v>-2.566201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3">
+        <v>-20.5285042</v>
+      </c>
+      <c r="D4" s="3">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-2.5660630000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3">
+        <v>-0.45238703000000002</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3">
+        <v>-0.22619300000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3">
+        <v>-0.59976622000000002</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2</v>
+      </c>
+      <c r="E6" s="3">
+        <v>2</v>
+      </c>
+      <c r="F6" s="3">
+        <v>-0.29988300000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3">
+        <v>-0.43872102000000002</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3">
+        <v>2</v>
+      </c>
+      <c r="F7" s="3">
+        <v>-0.21936</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="3">
+        <v>-20.634701369999998</v>
+      </c>
+      <c r="D8" s="3">
+        <v>8</v>
+      </c>
+      <c r="E8" s="3">
+        <v>8</v>
+      </c>
+      <c r="F8" s="3">
+        <v>-2.5793370000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="3">
+        <v>-20.634841980000001</v>
+      </c>
+      <c r="D9" s="3">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3">
+        <v>8</v>
+      </c>
+      <c r="F9" s="3">
+        <v>-2.5793550000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="3">
+        <v>-31.867761909999999</v>
+      </c>
+      <c r="D10" s="3">
+        <v>16</v>
+      </c>
+      <c r="E10" s="3">
+        <v>16</v>
+      </c>
+      <c r="F10" s="3">
+        <v>-1.991735</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="3">
+        <v>-0.27537549</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-0.27537499999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="3">
+        <v>-48.941790150000003</v>
+      </c>
+      <c r="D12" s="3">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3">
+        <v>4</v>
+      </c>
+      <c r="F12" s="3">
+        <v>-12.235447000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="3">
+        <v>-48.384432779999997</v>
+      </c>
+      <c r="D13" s="3">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3">
+        <v>4</v>
+      </c>
+      <c r="F13" s="3">
+        <v>-12.096107999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="3">
+        <v>-17.96539954</v>
+      </c>
+      <c r="D14" s="3">
+        <v>6</v>
+      </c>
+      <c r="E14" s="3">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3">
+        <v>-8.9826990000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="3">
+        <v>-131.3158286</v>
+      </c>
+      <c r="D15" s="3">
+        <v>33</v>
+      </c>
+      <c r="E15" s="3">
+        <v>11</v>
+      </c>
+      <c r="F15" s="3">
+        <v>-11.937802</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="3">
+        <v>-14.974708639999999</v>
+      </c>
+      <c r="D16" s="3">
+        <v>4</v>
+      </c>
+      <c r="E16" s="3">
+        <v>2</v>
+      </c>
+      <c r="F16" s="3">
+        <v>-7.4873539999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="3">
+        <v>-31.336455269999998</v>
+      </c>
+      <c r="D17" s="3">
+        <v>8</v>
+      </c>
+      <c r="E17" s="3">
+        <v>4</v>
+      </c>
+      <c r="F17" s="3">
+        <v>-7.8341130000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="3">
+        <v>-24.611714840000001</v>
+      </c>
+      <c r="D18" s="3">
+        <v>8</v>
+      </c>
+      <c r="E18" s="3">
+        <v>4</v>
+      </c>
+      <c r="F18" s="3">
+        <v>-6.1529280000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="3">
+        <v>-8.1522403499999996</v>
+      </c>
+      <c r="D19" s="3">
+        <v>4</v>
+      </c>
+      <c r="E19" s="3">
+        <v>2</v>
+      </c>
+      <c r="F19" s="3">
+        <v>-4.0761200000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="3">
+        <v>-11.90581793</v>
+      </c>
+      <c r="D20" s="3">
+        <v>4</v>
+      </c>
+      <c r="E20" s="3">
+        <v>2</v>
+      </c>
+      <c r="F20" s="3">
+        <v>-5.9529079999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="3">
+        <v>-141.58149359999999</v>
+      </c>
+      <c r="D21" s="3">
+        <v>28</v>
+      </c>
+      <c r="E21" s="3">
+        <v>4</v>
+      </c>
+      <c r="F21" s="3">
+        <v>-35.395372999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="3">
+        <v>-464.68080730000003</v>
+      </c>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24">
+        <v>-464.68099801</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="3">
+        <v>-457.96960819999998</v>
+      </c>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="3">
+        <v>-465.49424457999999</v>
+      </c>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F28" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3">
+        <v>-0.16729477200000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3">
+        <f>(C23-C26-F3+F9)/104</f>
+        <v>7.6950315384611495E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>